<commit_message>
feat: show coverage and quality in every report format (U6)
Excel, CSV, Markdown, and HTML reports now state each component family's
capture state (collected, collected empty, excluded, degraded, partial with
its expansion level, or unknown scope) and whether a quality audit ran, with
its verdict and issues.

A single pure helper, output/coverage.py, derives the rows and the quality
status; every writer renders from it.

- Excel: Coverage and Quality sheets after Summary. Existing sheets unchanged.
- CSV: <stem>.coverage.csv always, <stem>.quality_issues.csv when audited,
  quality verdict rows in summary.csv. Component CSVs unchanged.
- Markdown and HTML: Coverage and Quality sections after the header; empty
  component sections print the family's state instead of none.
- JSON is unchanged.

Sample outputs regenerated. .gitattributes marks sample CSV CRLF endings as
expected so git diff --check passes.
</commit_message>
<xml_diff>
--- a/sample_outputs/demo_prod.xlsx
+++ b/sample_outputs/demo_prod.xlsx
@@ -8,28 +8,31 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Dimensions" sheetId="2" r:id="rId2"/>
-    <sheet name="Metrics" sheetId="3" r:id="rId3"/>
-    <sheet name="Segments" sheetId="4" r:id="rId4"/>
-    <sheet name="Calculated Metrics" sheetId="5" r:id="rId5"/>
-    <sheet name="Virtual Report Suites" sheetId="6" r:id="rId6"/>
-    <sheet name="Classifications" sheetId="7" r:id="rId7"/>
+    <sheet name="Coverage" sheetId="2" r:id="rId2"/>
+    <sheet name="Quality" sheetId="3" r:id="rId3"/>
+    <sheet name="Dimensions" sheetId="4" r:id="rId4"/>
+    <sheet name="Metrics" sheetId="5" r:id="rId5"/>
+    <sheet name="Segments" sheetId="6" r:id="rId6"/>
+    <sheet name="Calculated Metrics" sheetId="7" r:id="rId7"/>
+    <sheet name="Virtual Report Suites" sheetId="8" r:id="rId8"/>
+    <sheet name="Classifications" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Calculated Metrics'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Classifications!$A$1:$D$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Dimensions!$A$1:$I$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Metrics!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Segments!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Calculated Metrics'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Classifications!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Coverage!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dimensions!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Metrics!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Segments!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Virtual Report Suites'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Virtual Report Suites'!$A$1:$I$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="105">
   <si>
     <t>Field</t>
   </si>
@@ -83,6 +86,24 @@
   </si>
   <si>
     <t>1.0.0</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Expansion Level</t>
+  </si>
+  <si>
+    <t>Collected</t>
+  </si>
+  <si>
+    <t>No quality audit ran.</t>
   </si>
   <si>
     <t>id</t>
@@ -332,16 +353,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -357,7 +370,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -365,30 +378,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -691,10 +686,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -793,6 +788,121 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -808,127 +918,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="C1" t="s">
         <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -937,7 +1047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -955,122 +1065,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="C1" t="s">
         <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H2" t="s">
-        <v>43</v>
-      </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" t="s">
         <v>51</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1079,7 +1189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1097,99 +1207,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>26</v>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>71</v>
+      </c>
+      <c r="J1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="J2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="K2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1198,7 +1308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1217,79 +1327,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s">
         <v>26</v>
+      </c>
+      <c r="I1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1298,7 +1408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1315,61 +1425,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>26</v>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1378,7 +1488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1390,31 +1500,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>26</v>
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: show coverage and quality in every report format (U6) (#155)
Excel, CSV, Markdown, and HTML reports now state each component family's
capture state (collected, collected empty, excluded, degraded, partial with
its expansion level, or unknown scope) and whether a quality audit ran, with
its verdict and issues.

A single pure helper, output/coverage.py, derives the rows and the quality
status; every writer renders from it.

- Excel: Coverage and Quality sheets after Summary. Existing sheets unchanged.
- CSV: <stem>.coverage.csv always, <stem>.quality_issues.csv when audited,
  quality verdict rows in summary.csv. Component CSVs unchanged.
- Markdown and HTML: Coverage and Quality sections after the header; empty
  component sections print the family's state instead of none.
- JSON is unchanged.

Sample outputs regenerated. .gitattributes marks sample CSV CRLF endings as
expected so git diff --check passes.
</commit_message>
<xml_diff>
--- a/sample_outputs/demo_prod.xlsx
+++ b/sample_outputs/demo_prod.xlsx
@@ -8,28 +8,31 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Dimensions" sheetId="2" r:id="rId2"/>
-    <sheet name="Metrics" sheetId="3" r:id="rId3"/>
-    <sheet name="Segments" sheetId="4" r:id="rId4"/>
-    <sheet name="Calculated Metrics" sheetId="5" r:id="rId5"/>
-    <sheet name="Virtual Report Suites" sheetId="6" r:id="rId6"/>
-    <sheet name="Classifications" sheetId="7" r:id="rId7"/>
+    <sheet name="Coverage" sheetId="2" r:id="rId2"/>
+    <sheet name="Quality" sheetId="3" r:id="rId3"/>
+    <sheet name="Dimensions" sheetId="4" r:id="rId4"/>
+    <sheet name="Metrics" sheetId="5" r:id="rId5"/>
+    <sheet name="Segments" sheetId="6" r:id="rId6"/>
+    <sheet name="Calculated Metrics" sheetId="7" r:id="rId7"/>
+    <sheet name="Virtual Report Suites" sheetId="8" r:id="rId8"/>
+    <sheet name="Classifications" sheetId="9" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Calculated Metrics'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Classifications!$A$1:$D$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Dimensions!$A$1:$I$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Metrics!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Segments!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Calculated Metrics'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Classifications!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Coverage!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dimensions!$A$1:$I$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Metrics!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Segments!$A$1:$K$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary!$A$1:$B$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Virtual Report Suites'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Virtual Report Suites'!$A$1:$I$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="105">
   <si>
     <t>Field</t>
   </si>
@@ -83,6 +86,24 @@
   </si>
   <si>
     <t>1.0.0</t>
+  </si>
+  <si>
+    <t>Family</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Expansion Level</t>
+  </si>
+  <si>
+    <t>Collected</t>
+  </si>
+  <si>
+    <t>No quality audit ran.</t>
   </si>
   <si>
     <t>id</t>
@@ -332,16 +353,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -357,7 +370,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -365,30 +378,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -691,10 +686,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -793,6 +788,121 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -808,127 +918,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="C1" t="s">
         <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="G2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I4" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G5" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="H5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="I5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -937,7 +1047,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -955,122 +1065,122 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="C1" t="s">
         <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" t="s">
         <v>49</v>
       </c>
-      <c r="B2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D2" t="s">
-        <v>56</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H2" t="s">
-        <v>43</v>
-      </c>
       <c r="I2" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E4" t="s">
+        <v>64</v>
+      </c>
+      <c r="F4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H4" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" t="s">
         <v>51</v>
-      </c>
-      <c r="B4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" t="s">
-        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1079,7 +1189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1097,99 +1207,99 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>26</v>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" t="s">
+        <v>70</v>
+      </c>
+      <c r="H1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" t="s">
+        <v>71</v>
+      </c>
+      <c r="J1" t="s">
+        <v>72</v>
+      </c>
+      <c r="K1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="G2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="J2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="K2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="G3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H3" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1198,7 +1308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1217,79 +1327,79 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="B1" t="s">
         <v>25</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s">
         <v>26</v>
+      </c>
+      <c r="I1" t="s">
+        <v>69</v>
+      </c>
+      <c r="J1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="I2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="K2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="L2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1298,7 +1408,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1315,61 +1425,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="A1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>26</v>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" t="s">
+        <v>72</v>
+      </c>
+      <c r="I1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="I2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1378,7 +1488,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1390,31 +1500,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>26</v>
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add readable definition summaries and a references appendix (U11)
Segments gain definition_summary and calculated metrics gain formula_summary, a one-line readable form of the definition built from a conservative subset of the AA 2.0 grammar. Nodes outside it show raw as [unparsed: <func>]. Both families gain metric_references and segment_references. The full definition JSON stays in every output.

A references appendix lists, for each calculated metric, segment, and virtual report suite, its direct references (resolved or unresolved against the capture) and what references it. It is an Excel References sheet, <stem>.references.csv, a Markdown and HTML section, and a top-level JSON references block.

The parser and resolver live in the pure module sdr/definitions.py with depth and size limits. JSON output is enriched at write time; snapshots keep the plain payload, so diffs are unaffected.
</commit_message>
<xml_diff>
--- a/sample_outputs/demo_prod.xlsx
+++ b/sample_outputs/demo_prod.xlsx
@@ -16,14 +16,16 @@
     <sheet name="Calculated Metrics" sheetId="7" r:id="rId7"/>
     <sheet name="Virtual Report Suites" sheetId="8" r:id="rId8"/>
     <sheet name="Classifications" sheetId="9" r:id="rId9"/>
+    <sheet name="References" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Calculated Metrics'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Calculated Metrics'!$A$1:$O$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Classifications!$A$1:$D$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Coverage!$A$1:$D$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Dimensions!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Metrics!$A$1:$J$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Segments!$A$1:$K$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">References!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Segments!$A$1:$N$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Summary!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Virtual Report Suites'!$A$1:$I$2</definedName>
   </definedNames>
@@ -32,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="127">
   <si>
     <t>Field</t>
   </si>
@@ -253,6 +255,15 @@
     <t>modified</t>
   </si>
   <si>
+    <t>definition_summary</t>
+  </si>
+  <si>
+    <t>metric_references</t>
+  </si>
+  <si>
+    <t>segment_references</t>
+  </si>
+  <si>
     <t>s_111</t>
   </si>
   <si>
@@ -271,10 +282,10 @@
     <t>42</t>
   </si>
   <si>
-    <t>{"container": {"context": "hits", "func": "container", "pred": {"func": "eq", "val": "mobile"}}, "version": [1, 0, 0]}</t>
-  </si>
-  <si>
-    <t>{"container": {"context": "visits", "func": "container", "pred": {"func": "eq", "val": "returning"}}, "version": [1, 0, 0]}</t>
+    <t>{"container": {"context": "hits", "func": "container", "pred": {"func": "streq", "str": "mobile", "val": {"func": "attr", "name": "variables/evar2"}}}, "func": "segment", "version": [1, 0, 0]}</t>
+  </si>
+  <si>
+    <t>{"container": {"context": "visits", "func": "container", "pred": {"func": "and", "preds": [{"func": "gt", "num": 1, "val": {"func": "attr", "name": "variables/visitnumber"}}, {"evt": {"func": "event", "name": "metrics/pageviews"}, "func": "event-exists"}]}}, "func": "segment", "version": [1, 0, 0]}</t>
   </si>
   <si>
     <t>2025-01-01T00:00:00Z</t>
@@ -283,12 +294,21 @@
     <t>2025-01-02T00:00:00Z</t>
   </si>
   <si>
+    <t>Hit where variables/evar2 = 'mobile'</t>
+  </si>
+  <si>
+    <t>Visit where variables/visitnumber &gt; 1 AND metrics/pageviews exists</t>
+  </si>
+  <si>
     <t>polarity</t>
   </si>
   <si>
     <t>categories</t>
   </si>
   <si>
+    <t>formula_summary</t>
+  </si>
+  <si>
     <t>cm_1</t>
   </si>
   <si>
@@ -307,12 +327,18 @@
     <t>decimal</t>
   </si>
   <si>
-    <t>{"formula": {"args": ["metrics/orders", "metrics/visits"], "func": "divide"}}</t>
+    <t>{"formula": {"col1": {"func": "metric", "name": "metrics/orders"}, "col2": {"func": "segment", "metric": {"func": "metric", "name": "metrics/visits"}, "segment_id": "s_222"}, "func": "divide"}, "func": "calc-metric", "version": [1, 0, 0]}</t>
   </si>
   <si>
     <t>["Conversion"]</t>
   </si>
   <si>
+    <t>metrics/orders / metrics/visits[segment s_222]</t>
+  </si>
+  <si>
+    <t>metrics/orders, metrics/visits</t>
+  </si>
+  <si>
     <t>parent_rsid</t>
   </si>
   <si>
@@ -347,6 +373,48 @@
   </si>
   <si>
     <t>Campaign Metadata</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Relation</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Target Family</t>
+  </si>
+  <si>
+    <t>Target ID</t>
+  </si>
+  <si>
+    <t>Target Name</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>references</t>
+  </si>
+  <si>
+    <t>referenced by</t>
+  </si>
+  <si>
+    <t>metric</t>
+  </si>
+  <si>
+    <t>segment</t>
+  </si>
+  <si>
+    <t>s_eu</t>
+  </si>
+  <si>
+    <t>resolved</t>
+  </si>
+  <si>
+    <t>unresolved</t>
   </si>
 </sst>
 </file>
@@ -787,6 +855,222 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="23.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.7109375" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G1" t="s">
+        <v>117</v>
+      </c>
+      <c r="H1" t="s">
+        <v>118</v>
+      </c>
+      <c r="I1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
+        <v>55</v>
+      </c>
+      <c r="H2" t="s">
+        <v>58</v>
+      </c>
+      <c r="I2" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
+        <v>122</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>57</v>
+      </c>
+      <c r="H3" t="s">
+        <v>60</v>
+      </c>
+      <c r="I3" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E4" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H4" t="s">
+        <v>79</v>
+      </c>
+      <c r="I4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" t="s">
+        <v>122</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>91</v>
+      </c>
+      <c r="H6" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G7" t="s">
+        <v>124</v>
+      </c>
+      <c r="I7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I7"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D7"/>
@@ -1191,7 +1475,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.7109375" customWidth="1"/>
@@ -1204,9 +1488,12 @@
     <col min="8" max="8" width="6.7109375" customWidth="1"/>
     <col min="9" max="10" width="22.7109375" customWidth="1"/>
     <col min="11" max="11" width="7.7109375" customWidth="1"/>
+    <col min="12" max="12" width="60.7109375" customWidth="1"/>
+    <col min="13" max="13" width="19.7109375" customWidth="1"/>
+    <col min="14" max="14" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1240,25 +1527,34 @@
       <c r="K1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="L1" t="s">
+        <v>73</v>
+      </c>
+      <c r="M1" t="s">
+        <v>74</v>
+      </c>
+      <c r="N1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="G2" t="s">
         <v>51</v>
@@ -1267,30 +1563,33 @@
         <v>49</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="J2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="K2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="L2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G3" t="s">
         <v>51</v>
@@ -1301,16 +1600,22 @@
       <c r="K3" t="s">
         <v>51</v>
       </c>
+      <c r="L3" t="s">
+        <v>87</v>
+      </c>
+      <c r="M3" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K3"/>
+  <autoFilter ref="A1:N3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -1324,9 +1629,12 @@
     <col min="10" max="10" width="6.7109375" customWidth="1"/>
     <col min="11" max="11" width="16.7109375" customWidth="1"/>
     <col min="12" max="12" width="7.7109375" customWidth="1"/>
+    <col min="13" max="13" width="48.7109375" customWidth="1"/>
+    <col min="14" max="14" width="32.7109375" customWidth="1"/>
+    <col min="15" max="15" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12">
+    <row r="1" spans="1:15">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1343,7 +1651,7 @@
         <v>68</v>
       </c>
       <c r="F1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="G1" t="s">
         <v>52</v>
@@ -1358,52 +1666,70 @@
         <v>31</v>
       </c>
       <c r="K1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="L1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:12">
+      <c r="M1" t="s">
+        <v>90</v>
+      </c>
+      <c r="N1" t="s">
+        <v>74</v>
+      </c>
+      <c r="O1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F2" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="G2" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H2" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="J2" t="s">
         <v>49</v>
       </c>
       <c r="K2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="L2" t="s">
         <v>51</v>
       </c>
+      <c r="M2" t="s">
+        <v>99</v>
+      </c>
+      <c r="N2" t="s">
+        <v>100</v>
+      </c>
+      <c r="O2" t="s">
+        <v>77</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:O2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1432,19 +1758,19 @@
         <v>25</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="D1" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s">
         <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="H1" t="s">
         <v>72</v>
@@ -1455,28 +1781,28 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B2" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="E2" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="F2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="G2" t="s">
         <v>49</v>
       </c>
       <c r="H2" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="I2" t="s">
         <v>51</v>
@@ -1515,10 +1841,10 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>

</xml_diff>